<commit_message>
reception layout and workflow fixes
</commit_message>
<xml_diff>
--- a/src/menu.database.xlsx
+++ b/src/menu.database.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maciejtokarz/BrunhollOrders/src/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CED314C-C773-5A4D-AF1A-DDB040D68FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Arkusz1" sheetId="1" r:id="rId5"/>
+    <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -169,9 +178,6 @@
     <t>chef_dessert</t>
   </si>
   <si>
-    <t>kitchen,bar</t>
-  </si>
-  <si>
     <t>Dessert</t>
   </si>
   <si>
@@ -566,22 +572,27 @@
   </si>
   <si>
     <t>11</t>
+  </si>
+  <si>
+    <t>Soup</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -589,35 +600,40 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -625,7 +641,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -815,17 +831,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:I69"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -854,7 +873,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -879,7 +898,7 @@
       <c r="H2" s="1"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -904,7 +923,7 @@
       <c r="H3" s="1"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -929,7 +948,7 @@
       <c r="H4" s="1"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
@@ -954,7 +973,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
@@ -979,7 +998,7 @@
       <c r="H6" s="1"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -1004,7 +1023,7 @@
       <c r="H7" s="1"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
@@ -1029,7 +1048,7 @@
       <c r="H8" s="1"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
@@ -1054,7 +1073,7 @@
       <c r="H9" s="1"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="1" t="s">
         <v>34</v>
       </c>
@@ -1079,7 +1098,7 @@
       <c r="H10" s="1"/>
       <c r="I10" s="2"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="1" t="s">
         <v>37</v>
       </c>
@@ -1087,13 +1106,13 @@
         <v>38</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>11</v>
+        <v>56</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>39</v>
+        <v>184</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>14</v>
@@ -1104,7 +1123,7 @@
       <c r="H11" s="1"/>
       <c r="I11" s="2"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1" t="s">
         <v>40</v>
       </c>
@@ -1129,7 +1148,7 @@
       <c r="H12" s="1"/>
       <c r="I12" s="2"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="1" t="s">
         <v>43</v>
       </c>
@@ -1154,7 +1173,7 @@
       <c r="H13" s="1"/>
       <c r="I13" s="2"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="1" t="s">
         <v>45</v>
       </c>
@@ -1179,7 +1198,7 @@
       <c r="H14" s="1"/>
       <c r="I14" s="2"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="1" t="s">
         <v>48</v>
       </c>
@@ -1204,7 +1223,7 @@
       <c r="H15" s="1"/>
       <c r="I15" s="2"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1" t="s">
         <v>50</v>
       </c>
@@ -1212,13 +1231,13 @@
         <v>51</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>14</v>
@@ -1229,21 +1248,21 @@
       <c r="H16" s="1"/>
       <c r="I16" s="2"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="C17" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>14</v>
@@ -1254,21 +1273,21 @@
       <c r="H17" s="1"/>
       <c r="I17" s="2"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="C18" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>14</v>
@@ -1279,21 +1298,21 @@
       <c r="H18" s="1"/>
       <c r="I18" s="2"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="C19" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>14</v>
@@ -1304,21 +1323,21 @@
       <c r="H19" s="1"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="C20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>14</v>
@@ -1329,71 +1348,71 @@
       <c r="H20" s="1"/>
       <c r="I20" s="2"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="2"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="C22" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="2"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="C23" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>14</v>
@@ -1402,25 +1421,25 @@
         <v>15</v>
       </c>
       <c r="H23" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I23" s="2"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="I23" s="2"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="C24" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>14</v>
@@ -1429,25 +1448,25 @@
         <v>18</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I24" s="2"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="C25" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>14</v>
@@ -1456,25 +1475,25 @@
         <v>21</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I25" s="2"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="C26" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>14</v>
@@ -1485,21 +1504,21 @@
       <c r="H26" s="1"/>
       <c r="I26" s="2"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="C27" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>14</v>
@@ -1510,21 +1529,21 @@
       <c r="H27" s="1"/>
       <c r="I27" s="2"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="C28" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D28" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>14</v>
@@ -1535,21 +1554,21 @@
       <c r="H28" s="1"/>
       <c r="I28" s="2"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="C29" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>14</v>
@@ -1560,96 +1579,96 @@
       <c r="H29" s="1"/>
       <c r="I29" s="2"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>90</v>
-      </c>
       <c r="C30" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="F30" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="2"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="2"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="C32" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D32" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="F32" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="2"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="C33" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>14</v>
@@ -1660,21 +1679,21 @@
       <c r="H33" s="1"/>
       <c r="I33" s="2"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="C34" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>14</v>
@@ -1685,21 +1704,21 @@
       <c r="H34" s="1"/>
       <c r="I34" s="2"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="C35" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>14</v>
@@ -1710,21 +1729,21 @@
       <c r="H35" s="1"/>
       <c r="I35" s="2"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="C36" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>14</v>
@@ -1735,21 +1754,21 @@
       <c r="H36" s="1"/>
       <c r="I36" s="2"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="C37" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>14</v>
@@ -1760,21 +1779,21 @@
       <c r="H37" s="1"/>
       <c r="I37" s="2"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="C38" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>14</v>
@@ -1785,21 +1804,21 @@
       <c r="H38" s="1"/>
       <c r="I38" s="2"/>
     </row>
-    <row r="39">
+    <row r="39" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>111</v>
-      </c>
       <c r="C39" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>14</v>
@@ -1810,21 +1829,21 @@
       <c r="H39" s="1"/>
       <c r="I39" s="2"/>
     </row>
-    <row r="40">
+    <row r="40" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="C40" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>14</v>
@@ -1835,21 +1854,21 @@
       <c r="H40" s="1"/>
       <c r="I40" s="2"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="C41" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>14</v>
@@ -1860,21 +1879,21 @@
       <c r="H41" s="1"/>
       <c r="I41" s="2"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="C42" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>14</v>
@@ -1885,21 +1904,21 @@
       <c r="H42" s="1"/>
       <c r="I42" s="2"/>
     </row>
-    <row r="43">
+    <row r="43" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B43" s="1" t="s">
-        <v>120</v>
-      </c>
       <c r="C43" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>14</v>
@@ -1910,21 +1929,21 @@
       <c r="H43" s="1"/>
       <c r="I43" s="2"/>
     </row>
-    <row r="44">
+    <row r="44" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>122</v>
-      </c>
       <c r="C44" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>14</v>
@@ -1935,46 +1954,46 @@
       <c r="H44" s="1"/>
       <c r="I44" s="2"/>
     </row>
-    <row r="45">
+    <row r="45" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="C45" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H45" s="1"/>
       <c r="I45" s="2"/>
     </row>
-    <row r="46">
+    <row r="46" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="C46" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>14</v>
@@ -1985,21 +2004,21 @@
       <c r="H46" s="1"/>
       <c r="I46" s="2"/>
     </row>
-    <row r="47">
+    <row r="47" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="C47" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E47" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>130</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>14</v>
@@ -2010,21 +2029,21 @@
       <c r="H47" s="1"/>
       <c r="I47" s="2"/>
     </row>
-    <row r="48">
+    <row r="48" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B48" s="1" t="s">
-        <v>132</v>
-      </c>
       <c r="C48" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>14</v>
@@ -2035,21 +2054,21 @@
       <c r="H48" s="1"/>
       <c r="I48" s="2"/>
     </row>
-    <row r="49">
+    <row r="49" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B49" s="1" t="s">
-        <v>134</v>
-      </c>
       <c r="C49" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>14</v>
@@ -2060,71 +2079,71 @@
       <c r="H49" s="1"/>
       <c r="I49" s="2"/>
     </row>
-    <row r="50">
+    <row r="50" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B50" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="C50" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>137</v>
       </c>
       <c r="H50" s="1"/>
       <c r="I50" s="2"/>
     </row>
-    <row r="51">
+    <row r="51" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B51" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="C51" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="H51" s="1"/>
       <c r="I51" s="2"/>
     </row>
-    <row r="52">
+    <row r="52" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>14</v>
@@ -2135,121 +2154,121 @@
       <c r="H52" s="1"/>
       <c r="I52" s="2"/>
     </row>
-    <row r="53">
+    <row r="53" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B53" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="C53" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="H53" s="1"/>
       <c r="I53" s="2"/>
     </row>
-    <row r="54">
+    <row r="54" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B54" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>146</v>
-      </c>
       <c r="C54" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H54" s="1"/>
       <c r="I54" s="2"/>
     </row>
-    <row r="55">
+    <row r="55" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="C55" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="H55" s="1"/>
       <c r="I55" s="2"/>
     </row>
-    <row r="56">
+    <row r="56" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B56" s="1" t="s">
-        <v>151</v>
-      </c>
       <c r="C56" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H56" s="1"/>
       <c r="I56" s="2"/>
     </row>
-    <row r="57">
+    <row r="57" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="C57" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E57" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>14</v>
@@ -2258,25 +2277,25 @@
         <v>15</v>
       </c>
       <c r="H57" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="I57" s="2"/>
+    </row>
+    <row r="58" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A58" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="I57" s="2"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="s">
+      <c r="B58" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="C58" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C58" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D58" s="1" t="s">
+      <c r="E58" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>14</v>
@@ -2287,21 +2306,21 @@
       <c r="H58" s="1"/>
       <c r="I58" s="2"/>
     </row>
-    <row r="59">
+    <row r="59" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B59" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="C59" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D59" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>14</v>
@@ -2312,21 +2331,21 @@
       <c r="H59" s="1"/>
       <c r="I59" s="2"/>
     </row>
-    <row r="60">
+    <row r="60" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B60" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="C60" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D60" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E60" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>14</v>
@@ -2337,21 +2356,21 @@
       <c r="H60" s="1"/>
       <c r="I60" s="2"/>
     </row>
-    <row r="61">
+    <row r="61" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A61" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B61" s="1" t="s">
-        <v>165</v>
-      </c>
       <c r="C61" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D61" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E61" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>14</v>
@@ -2362,96 +2381,96 @@
       <c r="H61" s="1"/>
       <c r="I61" s="2"/>
     </row>
-    <row r="62">
+    <row r="62" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A62" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B62" s="1" t="s">
-        <v>167</v>
-      </c>
       <c r="C62" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D62" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E62" s="1" t="s">
-        <v>159</v>
-      </c>
       <c r="F62" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H62" s="1"/>
       <c r="I62" s="2"/>
     </row>
-    <row r="63">
+    <row r="63" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A63" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="C63" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G63" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>170</v>
       </c>
       <c r="H63" s="1"/>
       <c r="I63" s="2"/>
     </row>
-    <row r="64">
+    <row r="64" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A64" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="B64" s="1" t="s">
-        <v>172</v>
-      </c>
       <c r="C64" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D64" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E64" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E64" s="1" t="s">
-        <v>159</v>
-      </c>
       <c r="F64" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H64" s="1"/>
       <c r="I64" s="2"/>
     </row>
-    <row r="65">
+    <row r="65" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A65" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="C65" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E65" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>175</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>14</v>
@@ -2462,21 +2481,21 @@
       <c r="H65" s="1"/>
       <c r="I65" s="2"/>
     </row>
-    <row r="66">
+    <row r="66" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A66" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B66" s="1" t="s">
-        <v>177</v>
-      </c>
       <c r="C66" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>14</v>
@@ -2487,12 +2506,12 @@
       <c r="H66" s="1"/>
       <c r="I66" s="2"/>
     </row>
-    <row r="67">
+    <row r="67" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A67" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>11</v>
@@ -2512,57 +2531,57 @@
       <c r="H67" s="1"/>
       <c r="I67" s="2"/>
     </row>
-    <row r="68">
+    <row r="68" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A68" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B68" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B68" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="C68" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E68" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D68" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="F68" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H68" s="1"/>
       <c r="I68" s="2"/>
     </row>
-    <row r="69">
+    <row r="69" spans="1:9" ht="13" x14ac:dyDescent="0.15">
       <c r="A69" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="C69" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E69" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F69" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G69" s="1" t="s">
-        <v>184</v>
       </c>
       <c r="H69" s="1"/>
       <c r="I69" s="2"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>